<commit_message>
Expand Agency Media Buying Blueprint to 12 operational tabs including Competitor Ad Hooks, Trending Audio, Tenant Co-Op Matching, Visual Photo Mining, 4-Year Rating Drift, and ManyChat FAQ Funnels
</commit_message>
<xml_diff>
--- a/lakeshore_agency_media_buying_blueprint.xlsx
+++ b/lakeshore_agency_media_buying_blueprint.xlsx
@@ -13,6 +13,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Creator Whitelisting Matrix" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Budget &amp; Unit Economics" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. UTM &amp; Attribution Governance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Competitor Ad Deconstruction" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Trending Audio Playlist" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Tenant Co-Op Ad Matching" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Visual Asset Photo Mining" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 4-Year Rating Drift" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. FAQ &amp; ManyChat DM Funnel" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,7 +65,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +97,11 @@
         <fgColor rgb="00FCF3CF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -118,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -176,6 +187,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -888,6 +908,737 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CUSTOMER PHOTO MINING: WHAT 15,000+ SHOPPERS PHOTOGRAPH &amp; HOW TO MONETIZE IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Shopper Photo Category</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>% Share of Total Photos</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Primary Subject Photographed</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Shopper Motivation / Trigger</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>KOPA On-Ground Infrastructure Action</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Paid UGC Ad Campaign Idea</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>🍽️ Food &amp; Cocktail Plating</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>42% of all photos</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Smoked cocktails, sushi platters, artisanal pasta, dessert presentations</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Status sharing on Instagram Stories &amp; food review flex</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Install warm ring lighting &amp; photogenic table decor in all dining zones</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Run '#KopaBites' monthly contest with ₹10,000 dining vouchers for top UGC reel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>🪞 Mirror Selfies &amp; OOTD</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>28% of all photos</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Full-length mirror selfies in luxury restrooms and elevator lobbies</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Outfit flex, hair &amp; makeup showcase before date night/events</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Build dedicated 'Infinity Mirrors' with perfect flattering lighting &amp; branded decal</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Turn best customer mirror selfies into Meta Carousel testimonial ads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>🏛️ Atrium &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>16% of all photos</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Open-air sky views, water fountains, festive light chandeliers</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic appreciation of modern non-chaotic mall design</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Ensure landscape plants, natural sunlight corridors are pristine 24/7</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Run 4K slow-mo B-roll ads targeting architecture and interior design enthusiasts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>🚗 Parking Receipts &amp; Clamped Tires</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>14% of all photos</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Phoenix Marketcity ₹150 parking slips, wheel clamp notices, exit line gridlock</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Negative venting and consumer anger on Google Maps</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Maintain zero-friction valet parking &amp; prominently display free valet with ₹2k spend</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Feature split screen ad: Competitor ₹150 parking slip vs KOPA complimentary valet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HISTORICAL RATING DRIFT ANALYSIS (2023 - 2026): COMPETITOR DECAY VS KOPA ASCENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mall Name</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2023 Avg Rating</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2024 Avg Rating</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2025 Avg Rating</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026 Live Rating</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>3-Year Trend Drift</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Core Operational Driver of Trend</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>Phoenix Avenue of Stars (Pune)</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>4.69 ★ (278)</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>4.56 ★ (187)</t>
+        </is>
+      </c>
+      <c r="E3" s="21" t="inlineStr">
+        <is>
+          <t>4.47 ★ (317)</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>3.92 ★ (367)</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="inlineStr">
+        <is>
+          <t>🔻 -0.77★ (Severe Decay)</t>
+        </is>
+      </c>
+      <c r="H3" s="22" t="inlineStr">
+        <is>
+          <t>Nagar road metro construction + aggressive parking fees + basement congestion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>KOPA Mall Pune (Lake Shore)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>N/A (Pre-Launch)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>4.36 ★ (491)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>4.45 ★ (1,066)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>4.44 ★ (808)</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>🟢 +0.08★ (Rising Stability)</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Steady retail occupancy, fine dining maturation, and valet satisfaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>The Pavillion Pune</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>4.60 ★ (Est)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>4.58 ★ (Est)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>4.53 ★ (1,456)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>4.52 ★ (1,034)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>🔻 -0.08★ (Stagnant)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Stable Central Pune footfall but limited high-end brand expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Amanora Mall Pune</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>4.65 ★ (Est)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>4.60 ★ (Est)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>4.62 ★ (157)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>4.51 ★ (1,443)</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>🔻 -0.14★ (Minor Decline)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Sprawling layout fatigue and competition from newer Kharadi developments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Lulu Mall Hyderabad (Y Junction)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>N/A (Pre-Launch)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>4.45 ★ (Est)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>4.26 ★ (1,212)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>4.18 ★ (2,608)</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>🔻 -0.27★ (Crowd Friction)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Overwhelming weekend crowd density, long billing lines, and parking delays.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INSTAGRAM MANYCHAT AUTOMATION FUNNEL: MINED FROM 1,524 REAL SHOPPER INQUIRIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Customer Comment Trigger Keyword</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Underlying Shopper Intent</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Real Scraped Comment Example</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Automated ManyChat DM Response</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Call to Action Link in DM</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Conversion Goal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Comments 'Location' or 'Address'</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Navigation &amp; Commute</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>"Where is this mall located? Is it near Koregaon Park?"</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>"Hey {First_Name}! ✨ KOPA is located in the heart of Koregaon Park, Pune. Click below for instant Google Maps directions &amp; valet access!"</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Google Maps PIN Link</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Footfall Visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Comments 'Valet' or 'Parking'</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Parking Friction Query</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>"How much are parking charges? Is valet available on weekends?"</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>"Hi {First_Name}! 🚗 Yes, KOPA offers seamless VIP Valet Parking right at the main entrance. Complimentary valet on shopping above ₹2,000!"</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Valet Digital Pass</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Zero-Friction Arrival</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Comments 'Pets' or 'Dog'</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Pet-Friendly Policy</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>"Are dogs allowed inside the mall? Looking for pet friendly places."</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>"Hi {First_Name}! 🐾 Yes, KOPA is 100% pet-friendly in our open-air plazas and outdoor dining cafes! We even have water bowls ready for your furry friend."</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Pet Guidelines &amp; Cafes Link</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Lifestyle Community Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Comments 'Table' or 'Dinner'</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>F&amp;B Table Booking</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>"Which rooftop restaurant is this? Need to book for anniversary tonight."</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>"Hey {First_Name}! 🍸 This is from our rooftop dining terrace at KOPA. Here is your direct VIP reservation link to skip the weekend waitlist!"</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Zomato Dineout VIP Link</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Table Reservation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Comments 'Movie' or 'PVR'</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Cinema Ticket Intent</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>"Is this the new PVR Director's Cut? How to book recliner seats?"</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>"Hi {First_Name}! 🎬 Yes! PVR Director's Cut at KOPA features luxury recliners and in-theatre gourmet dining. Tap below to book your seats on BookMyShow."</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>BookMyShow Direct Film Link</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Ticket Sale Conversion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2274,4 +3025,817 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>COMPETITOR META AD REVERSE-ENGINEERING: 425 ADS ANALYZED FOR HOOKS, FORMATS &amp; STRATEGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Advertiser / Mall Target</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ad Type / Hook Category</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Actual Scraped Ad Hook (0-3s Headline)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Dominant CTA</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Competitor Strategy Observed</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Vulnerability / Flaw in Competitor Ad</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>KOPA Counter-Strike Ad Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Phoenix Avenue Of Stars (Phoenix Pune)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Live Concert &amp; Event Hook</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>"🎤✨ The undisputed king of 90s nostalgia and soulful Qawwali is coming to Pune!"</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Uses massive celebrity concerts to generate footfall surges on Saturday nights.</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Creates severe parking bottlenecks (30-45 min queues) and gridlocks Nagar Road.</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Run geofenced dark ads to concert attendees leaving Phoenix: "Tired of concert parking traffic? Unwind with late-night cocktails at KOPA Koregaon Park — 5 mins away."</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Samsung (Inside Phoenix Marketcity)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Tenant Product Launch</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>"The all-new Galaxy Z Fold8 Ultra and Fold8. Own now, starting at ₹ 4500/month.* Visit Samsung Experience Store, Phoenix."</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Sign Up</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Tech brand co-funds store visit ads targeting gadget enthusiasts in Viman Nagar.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Generic corporate tech template; lacks luxury lifestyle context or VIP experience.</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Partner with Samsung/Apple at KOPA for a 'VIP Tech Lounge' experience ad targeting Boat Club Rd HNIs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Paul Cafe (Inside Phoenix Marketcity)</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>F&amp;B Break Hook</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>"🛍️🥮☕️ A much needed break in between shopping!! PAUL CAFE, Phoenix Marketcity Pune. A delightful open space…"</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Promotes quiet coffee retreat inside a chaotic mass mall.</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Shoppers still have to navigate noisy, crowded corridors to reach the cafe.</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>Position KOPA's entire open-air campus as the sanctuary: "Why search for a quiet corner in a loud mall? KOPA is designed as a tranquil luxury oasis from entrance to rooftop."</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Kohinoor / Godrej / Rohan Builders</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Catchment Proximity Real Estate</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>"📍 Viman Nagar – Near Phoenix Marketcity 🏡 2 &amp; 3 BHK Homes ₹1.05 Cr* – Happening Kharadi / Viman Nagar."</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Real estate developers spend ₹500K+/mo piggybacking on mall brand equity to sell luxury apartments.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Shows huge concentration of affluent homebuyers (₹1 Cr+ budgets) moving into East Pune.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Geofence new luxury housing societies (Kohinoor Kaleido, Godrej Ivara) with 'Welcome to the Neighborhood' KOPA privilege shopping passes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Lulu Mall Hyderabad (Y Junction)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Hypermarket EOSS Discount</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>"Mega Weekend Savings! Flat 50% off on electronics, grocery and fashion at Lulu Hypermarket."</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Shop Now</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Discount-driven mass footfall strategy attracting extreme crowd density.</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Causes 45-min checkout queues, parking chaos, and drives away affluent luxury shoppers.</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Lake Shore Y Junction counter-positioning: "Skip the hypermarket madness. Premium boutique retail, quick parking &amp; hassle-free weekend shopping at Y Junction."</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TRENDING AUDIO &amp; VIRALITY PLAYLIST: 15 HIGH-RETENTION TRACKS MINED FROM 4,076 REELS (230M+ VIEWS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Track Title &amp; Artist</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Total Scraped Views</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Reel Usage Count</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Vibe / Aesthetic Category</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Recommended Content Format for KOPA</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Algorithm Virality Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Sirius - Flow Loris</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>2,559,254 Views</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>⚡ High-Energy Luxury Beat</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Fast-cut transition reel showcasing luxury fashion try-ons (Armani, Mango, Sephora)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>🔥 98/100 (Top Virality)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Classical Romantic - StudioMaxMusic</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>2,522,296 Views</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>🎻 Quiet Luxury / Ambient Elegance</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Slow cinematic 4K drone &amp; gimbal pan of KOPA's open-air architecture &amp; natural light</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>⭐ 95/100 (High Retention)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Gimme More (Remix) - Britney / Remix</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>2,525,943 Views</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>✨ Glamour &amp; Nightlife</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Rooftop cocktail pouring, evening lighting, high-heels walking into dining lounge</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>🔥 96/100 (High Shares)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Pardesiya (Param Sundari) - Sachin-Jigar</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>2,279,180 Views</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>🪔 Festive &amp; Ethnic Luxury</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Diwali / Festive ethnic wear lookbooks (Tira, Ritu Kumar, designer festive drops)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>⭐ 94/100 (Seasonal Peak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Potter Waltz - Prague Philharmonic</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>2,278,800 Views</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>☕ Sophisticated Cafe &amp; Date-Night</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Artisanal coffee pours, French bakery desserts, quiet book-reading aesthetic</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>⭐ 92/100 (High Saves)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Ilahi (Reprise) - Mohit Chauhan / Pritam</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>2,061,598 Views</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>🌟 Nostalgic Youth / Weekend Chill</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Friends exploring KOPA, gelato tasting, PVR Director's Cut ticket booking</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>🔥 95/100 (High Engagement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Europe - HeartDrumMachine</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>1,867,695 Views</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>🏙️ Modern Architectural B-Roll</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Golden hour sun reflections on KOPA glass facades and minimalist water features</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>⭐ 90/100 (Aesthetic Niche)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TENANT BRAND CO-OP AD ENGINE: CO-FUNDED PAID AD CAMPAIGNS WITH ANCHOR BRANDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Anchor Tenant Brand</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Retail Category</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Co-Op Budget Match Ratio</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Tenant Campaign Angle</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Lake Shore Value Add</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Target ROAS / Footfall KPI</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Estimated Monthly Co-Op Spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Sephora &amp; Tira Beauty</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Luxury Beauty &amp; Skincare</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>1:1 Budget Match (50% Tenant / 50% KOPA)</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Exclusive masterclass invitations &amp; fragrance try-ons</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Geofence 5km around Koregaon Park &amp; Boat Club Road</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>₹120 CAC per in-store consultation</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>₹ 150,000 / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Armani Exchange &amp; Mango</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Premium Fashion</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1:1 Budget Match</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal Collection Launch &amp; VIP Styling appointments</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Whitelisted ads via top Pune fashion creators</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>3.5x ROAS on in-store billing</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>₹ 200,000 / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>PVR Director's Cut</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Ultra-Luxury Cinema</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>60% Tenant / 40% KOPA</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Dine-in Cinema &amp; Recliner Booking promos</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Meta Dark Ads targeting couples on Wed-Sun evenings</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>85%+ Weekend Recliner Occupancy</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>₹ 120,000 / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Gourmet Rooftop Restaurants</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Fine Dining &amp; Cocktails</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>50% Restaurant / 50% KOPA</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Weekend Table Reservation &amp; Signature Cocktail showcases</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Direct Zomato/Dineout instant booking link integration</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>600+ monthly table reservations</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="inlineStr">
+        <is>
+          <t>₹ 100,000 / month</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>